<commit_message>
chore(preprocessing): add project code for the preprocessing module
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="112">
   <si>
     <t xml:space="preserve">Project Information</t>
   </si>
@@ -51,6 +51,9 @@
     <t xml:space="preserve">Comments (Optional)</t>
   </si>
   <si>
+    <t xml:space="preserve">The Ready-made local ML models are: Farasa Segmenter, CAMeL Tools (Morphological Analyzer, MLE Disambiguator).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Modules (you can add new rows if needed)</t>
   </si>
   <si>
@@ -84,6 +87,18 @@
     <t xml:space="preserve">Design (UI/UX) is original work, Code is AI-generated</t>
   </si>
   <si>
+    <t xml:space="preserve">Preprocessing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The first module in our pipeline that does normalization, segmentation, and morphological analysis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NWS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predicts and suggests accurate Arabic words in near real-time as the user types using a hybrid machine learning pipeline.</t>
+  </si>
+  <si>
     <t xml:space="preserve">File Path (Relative to the Project Root, Glob patterns are allowed)</t>
   </si>
   <si>
@@ -262,6 +277,39 @@
   </si>
   <si>
     <t xml:space="preserve">Frontend deployment configuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/orchestrator.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part of preprocessing code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/schemas.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/utils/normalizer.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/utils/boundary.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/features/segmenter.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We use Farasa Segmenter inside it, but we customize the output to implement our own logic too</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/features/analyzer.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAMeL Tools (Morph Analyzer and MLE Disambiguator) were used in it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/preprocessing/notebooks/explore_libraries.ipynb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A notebook to explore the external libraries</t>
   </si>
   <si>
     <t xml:space="preserve">File Source</t>
@@ -461,7 +509,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,6 +571,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -856,7 +908,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="150.63"/>
@@ -904,25 +956,27 @@
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5"/>
+      <c r="B6" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>8</v>
@@ -930,39 +984,52 @@
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
       <c r="D12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10"/>
-      <c r="C13" s="11"/>
+      <c r="A13" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -998,7 +1065,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E1048576"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="91.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21"/>
@@ -1009,16 +1076,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>8</v>
@@ -1026,446 +1093,529 @@
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>35</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>61</v>
-      </c>
       <c r="D24" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B26" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="15" t="s">
-        <v>15</v>
-      </c>
       <c r="D26" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B27" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="15" t="s">
-        <v>15</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B29" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="15" t="s">
-        <v>15</v>
-      </c>
       <c r="D29" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="14"/>
+      <c r="A30" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="14"/>
+      <c r="A31" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="14"/>
+      <c r="A32" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="14"/>
+      <c r="A33" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="14"/>
+      <c r="A34" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="14"/>
+      <c r="A35" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="14"/>
+      <c r="A36" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="14"/>
@@ -4375,7 +4525,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="53.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="122.47"/>
@@ -4383,66 +4533,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4450,47 +4600,47 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(project-code): update the project code
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="124">
   <si>
     <t xml:space="preserve">Project Information</t>
   </si>
@@ -180,6 +180,9 @@
     <t xml:space="preserve">src/services/ged/evaluation/*.py</t>
   </si>
   <si>
+    <t xml:space="preserve">Generated by LLM</t>
+  </si>
+  <si>
     <t xml:space="preserve">src/services/ged/notebooks/*</t>
   </si>
   <si>
@@ -192,9 +195,6 @@
     <t xml:space="preserve">tests/services/ged/*</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by LLM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ged tests</t>
   </si>
   <si>
@@ -310,6 +310,42 @@
   </si>
   <si>
     <t xml:space="preserve">A notebook to explore the external libraries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/orchestrator.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part of NWS code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/schemas.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/features/cache/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/features/nwp/hybrid/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/features/nwp/lstm/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSTM model generated to use with another original model in a hybrid model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/features/nwp/word_ngram/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/services/nws/features/wac/char_ngram/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/services/nws/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test cases for the nws module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/services/preprocessing/*</t>
   </si>
   <si>
     <t xml:space="preserve">File Source</t>
@@ -1290,7 +1326,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>29</v>
@@ -1298,7 +1334,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>14</v>
@@ -1312,7 +1348,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>14</v>
@@ -1321,18 +1357,18 @@
         <v>37</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>57</v>
@@ -1346,7 +1382,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>59</v>
@@ -1360,7 +1396,7 @@
         <v>17</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>61</v>
@@ -1618,31 +1654,130 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="14"/>
+      <c r="A37" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="14"/>
+      <c r="A38" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="14"/>
+      <c r="A39" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="14"/>
+      <c r="A40" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="14"/>
+      <c r="A41" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="14"/>
+      <c r="A42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="14"/>
+      <c r="A43" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="14"/>
+      <c r="A44" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="14"/>
+      <c r="A45" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="14"/>
@@ -4533,10 +4668,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4544,7 +4679,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4552,7 +4687,7 @@
         <v>66</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4560,15 +4695,15 @@
         <v>37</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4576,23 +4711,23 @@
         <v>40</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4600,15 +4735,15 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4616,7 +4751,7 @@
         <v>40</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4624,7 +4759,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4632,7 +4767,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4640,7 +4775,7 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>